<commit_message>
Add Ex5B to week-01
</commit_message>
<xml_diff>
--- a/week-01/techsupply_dataset1.xlsx
+++ b/week-01/techsupply_dataset1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sguer\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED436E4C-B857-4F81-B4A4-BD3F9A95F794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15329B4C-AC11-4CB2-A025-77D1A950C93C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1103" yWindow="1103" windowWidth="16485" windowHeight="12060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sales_Data" sheetId="1" r:id="rId1"/>
@@ -1075,6 +1075,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:K301"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -1193,7 +1194,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2208</v>
       </c>
@@ -1263,7 +1264,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>2134</v>
       </c>
@@ -1298,7 +1299,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>2077</v>
       </c>
@@ -1368,7 +1369,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>2229</v>
       </c>
@@ -1403,7 +1404,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>2001</v>
       </c>
@@ -1438,7 +1439,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>2109</v>
       </c>
@@ -1473,7 +1474,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>2003</v>
       </c>
@@ -1543,7 +1544,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>2202</v>
       </c>
@@ -1613,7 +1614,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>2032</v>
       </c>
@@ -1753,7 +1754,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>2247</v>
       </c>
@@ -1788,7 +1789,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>2076</v>
       </c>
@@ -1823,7 +1824,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>2073</v>
       </c>
@@ -1858,7 +1859,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>2293</v>
       </c>
@@ -1893,7 +1894,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>2113</v>
       </c>
@@ -1928,7 +1929,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>2097</v>
       </c>
@@ -1963,7 +1964,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>2275</v>
       </c>
@@ -1998,7 +1999,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>2286</v>
       </c>
@@ -2068,7 +2069,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>2294</v>
       </c>
@@ -2103,7 +2104,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A30">
         <v>2031</v>
       </c>
@@ -2138,7 +2139,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A31">
         <v>2088</v>
       </c>
@@ -2173,7 +2174,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>2159</v>
       </c>
@@ -2243,7 +2244,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A34">
         <v>2219</v>
       </c>
@@ -2278,7 +2279,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A35">
         <v>2206</v>
       </c>
@@ -2313,7 +2314,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A36">
         <v>2010</v>
       </c>
@@ -2348,7 +2349,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A37">
         <v>2121</v>
       </c>
@@ -2383,7 +2384,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A38">
         <v>2069</v>
       </c>
@@ -2418,7 +2419,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A39">
         <v>2095</v>
       </c>
@@ -2453,7 +2454,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A40">
         <v>2222</v>
       </c>
@@ -2558,7 +2559,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A43">
         <v>2037</v>
       </c>
@@ -2593,7 +2594,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A44">
         <v>2161</v>
       </c>
@@ -2628,7 +2629,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A45">
         <v>2115</v>
       </c>
@@ -2663,7 +2664,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A46">
         <v>2155</v>
       </c>
@@ -2838,7 +2839,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A51">
         <v>2017</v>
       </c>
@@ -2873,7 +2874,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A52">
         <v>2080</v>
       </c>
@@ -2908,7 +2909,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A53">
         <v>2006</v>
       </c>
@@ -2943,7 +2944,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A54">
         <v>2036</v>
       </c>
@@ -2978,7 +2979,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A55">
         <v>2014</v>
       </c>
@@ -3013,7 +3014,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A56">
         <v>2207</v>
       </c>
@@ -3118,7 +3119,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A59">
         <v>2175</v>
       </c>
@@ -3188,7 +3189,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A61">
         <v>2236</v>
       </c>
@@ -3223,7 +3224,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A62">
         <v>2068</v>
       </c>
@@ -3293,7 +3294,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A64">
         <v>2078</v>
       </c>
@@ -3363,7 +3364,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A66">
         <v>2133</v>
       </c>
@@ -3503,7 +3504,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A70">
         <v>2197</v>
       </c>
@@ -3538,7 +3539,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A71">
         <v>2149</v>
       </c>
@@ -3573,7 +3574,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A72">
         <v>2264</v>
       </c>
@@ -3643,7 +3644,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A74">
         <v>2135</v>
       </c>
@@ -3678,7 +3679,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A75">
         <v>2099</v>
       </c>
@@ -3713,7 +3714,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A76">
         <v>2124</v>
       </c>
@@ -3748,7 +3749,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A77">
         <v>2246</v>
       </c>
@@ -3818,7 +3819,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A79">
         <v>2279</v>
       </c>
@@ -3853,7 +3854,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A80">
         <v>2274</v>
       </c>
@@ -3888,7 +3889,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A81">
         <v>2064</v>
       </c>
@@ -3923,7 +3924,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A82">
         <v>2118</v>
       </c>
@@ -3993,7 +3994,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A84">
         <v>2227</v>
       </c>
@@ -4063,7 +4064,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A86">
         <v>2257</v>
       </c>
@@ -4098,7 +4099,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A87">
         <v>2147</v>
       </c>
@@ -4133,7 +4134,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A88">
         <v>2261</v>
       </c>
@@ -4203,7 +4204,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A90">
         <v>2199</v>
       </c>
@@ -4238,7 +4239,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A91">
         <v>2122</v>
       </c>
@@ -4308,7 +4309,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A93">
         <v>2176</v>
       </c>
@@ -4343,7 +4344,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A94">
         <v>2075</v>
       </c>
@@ -4413,7 +4414,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A96">
         <v>2282</v>
       </c>
@@ -4448,7 +4449,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A97">
         <v>2125</v>
       </c>
@@ -4518,7 +4519,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A99">
         <v>2042</v>
       </c>
@@ -4553,7 +4554,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A100">
         <v>2072</v>
       </c>
@@ -4588,7 +4589,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A101">
         <v>2268</v>
       </c>
@@ -4693,7 +4694,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A104">
         <v>2217</v>
       </c>
@@ -4728,7 +4729,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A105">
         <v>2284</v>
       </c>
@@ -4798,7 +4799,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A107">
         <v>2234</v>
       </c>
@@ -4868,7 +4869,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A109">
         <v>2164</v>
       </c>
@@ -4938,7 +4939,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A111">
         <v>2276</v>
       </c>
@@ -4973,7 +4974,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A112">
         <v>2210</v>
       </c>
@@ -5008,7 +5009,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A113">
         <v>2262</v>
       </c>
@@ -5043,7 +5044,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A114">
         <v>2223</v>
       </c>
@@ -5113,7 +5114,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A116">
         <v>2251</v>
       </c>
@@ -5148,7 +5149,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A117">
         <v>2233</v>
       </c>
@@ -5218,7 +5219,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A119">
         <v>2038</v>
       </c>
@@ -5253,7 +5254,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A120">
         <v>2090</v>
       </c>
@@ -5323,7 +5324,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A122">
         <v>2204</v>
       </c>
@@ -5393,7 +5394,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A124">
         <v>2126</v>
       </c>
@@ -5428,7 +5429,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A125">
         <v>2299</v>
       </c>
@@ -5533,7 +5534,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A128">
         <v>2195</v>
       </c>
@@ -5603,7 +5604,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A130">
         <v>2187</v>
       </c>
@@ -5638,7 +5639,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A131">
         <v>2291</v>
       </c>
@@ -5673,7 +5674,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="132" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A132">
         <v>2171</v>
       </c>
@@ -5708,7 +5709,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="133" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A133">
         <v>2265</v>
       </c>
@@ -5743,7 +5744,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="134" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A134">
         <v>2250</v>
       </c>
@@ -5778,7 +5779,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="135" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A135">
         <v>2094</v>
       </c>
@@ -5813,7 +5814,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="136" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A136">
         <v>2030</v>
       </c>
@@ -5848,7 +5849,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A137">
         <v>2289</v>
       </c>
@@ -5918,7 +5919,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A139">
         <v>2170</v>
       </c>
@@ -6163,7 +6164,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A146">
         <v>2252</v>
       </c>
@@ -6198,7 +6199,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="147" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A147">
         <v>2152</v>
       </c>
@@ -6268,7 +6269,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A149">
         <v>2190</v>
       </c>
@@ -6303,7 +6304,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A150">
         <v>2084</v>
       </c>
@@ -6338,7 +6339,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="151" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A151">
         <v>2213</v>
       </c>
@@ -6373,7 +6374,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="152" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A152">
         <v>2057</v>
       </c>
@@ -6443,7 +6444,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A154">
         <v>2179</v>
       </c>
@@ -6478,7 +6479,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A155">
         <v>2181</v>
       </c>
@@ -6513,7 +6514,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A156">
         <v>2191</v>
       </c>
@@ -6583,7 +6584,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="158" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A158">
         <v>2254</v>
       </c>
@@ -6618,7 +6619,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="159" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A159">
         <v>2008</v>
       </c>
@@ -6653,7 +6654,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="160" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A160">
         <v>2218</v>
       </c>
@@ -6688,7 +6689,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="161" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A161">
         <v>2058</v>
       </c>
@@ -6723,7 +6724,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="162" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A162">
         <v>2013</v>
       </c>
@@ -6758,7 +6759,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="163" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A163">
         <v>2259</v>
       </c>
@@ -6793,7 +6794,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="164" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A164">
         <v>2277</v>
       </c>
@@ -6933,7 +6934,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A168">
         <v>2255</v>
       </c>
@@ -7003,7 +7004,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A170">
         <v>2039</v>
       </c>
@@ -7038,7 +7039,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="171" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A171">
         <v>2156</v>
       </c>
@@ -7073,7 +7074,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="172" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A172">
         <v>2145</v>
       </c>
@@ -7108,7 +7109,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="173" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A173">
         <v>2144</v>
       </c>
@@ -7143,7 +7144,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="174" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A174">
         <v>2196</v>
       </c>
@@ -7178,7 +7179,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="175" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A175">
         <v>2297</v>
       </c>
@@ -7248,7 +7249,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="177" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A177">
         <v>2049</v>
       </c>
@@ -7283,7 +7284,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="178" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A178">
         <v>2083</v>
       </c>
@@ -7318,7 +7319,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="179" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A179">
         <v>2258</v>
       </c>
@@ -7423,7 +7424,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="182" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A182">
         <v>2137</v>
       </c>
@@ -7458,7 +7459,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="183" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A183">
         <v>2167</v>
       </c>
@@ -7668,7 +7669,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="189" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A189">
         <v>2114</v>
       </c>
@@ -7703,7 +7704,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="190" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A190">
         <v>2146</v>
       </c>
@@ -7738,7 +7739,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="191" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A191">
         <v>2281</v>
       </c>
@@ -7773,7 +7774,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="192" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A192">
         <v>2221</v>
       </c>
@@ -7808,7 +7809,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="193" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A193">
         <v>2065</v>
       </c>
@@ -7843,7 +7844,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="194" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A194">
         <v>2104</v>
       </c>
@@ -7878,7 +7879,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="195" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A195">
         <v>2029</v>
       </c>
@@ -7913,7 +7914,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="196" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A196">
         <v>2016</v>
       </c>
@@ -7948,7 +7949,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="197" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A197">
         <v>2101</v>
       </c>
@@ -7983,7 +7984,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="198" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A198">
         <v>2105</v>
       </c>
@@ -8018,7 +8019,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="199" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A199">
         <v>2127</v>
       </c>
@@ -8053,7 +8054,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="200" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A200">
         <v>2278</v>
       </c>
@@ -8123,7 +8124,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="202" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="202" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A202">
         <v>2091</v>
       </c>
@@ -8158,7 +8159,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="203" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="203" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A203">
         <v>2230</v>
       </c>
@@ -8193,7 +8194,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="204" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="204" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A204">
         <v>2269</v>
       </c>
@@ -8228,7 +8229,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="205" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="205" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A205">
         <v>2185</v>
       </c>
@@ -8263,7 +8264,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="206" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="206" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A206">
         <v>2138</v>
       </c>
@@ -8298,7 +8299,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="207" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="207" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A207">
         <v>2271</v>
       </c>
@@ -8333,7 +8334,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="208" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="208" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A208">
         <v>2022</v>
       </c>
@@ -8368,7 +8369,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="209" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="209" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A209">
         <v>2248</v>
       </c>
@@ -8403,7 +8404,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="210" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="210" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A210">
         <v>2044</v>
       </c>
@@ -8438,7 +8439,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="211" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="211" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A211">
         <v>2002</v>
       </c>
@@ -8473,7 +8474,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="212" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="212" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A212">
         <v>2300</v>
       </c>
@@ -8508,7 +8509,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="213" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="213" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A213">
         <v>2225</v>
       </c>
@@ -8543,7 +8544,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="214" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="214" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A214">
         <v>2270</v>
       </c>
@@ -8578,7 +8579,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="215" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="215" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A215">
         <v>2117</v>
       </c>
@@ -8613,7 +8614,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="216" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="216" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A216">
         <v>2024</v>
       </c>
@@ -8648,7 +8649,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="217" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="217" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A217">
         <v>2240</v>
       </c>
@@ -8683,7 +8684,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="218" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="218" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A218">
         <v>2020</v>
       </c>
@@ -8718,7 +8719,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="219" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="219" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A219">
         <v>2009</v>
       </c>
@@ -8753,7 +8754,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="220" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="220" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A220">
         <v>2238</v>
       </c>
@@ -8788,7 +8789,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="221" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="221" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A221">
         <v>2174</v>
       </c>
@@ -8858,7 +8859,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="223" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="223" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A223">
         <v>2055</v>
       </c>
@@ -8893,7 +8894,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="224" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="224" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A224">
         <v>2110</v>
       </c>
@@ -8928,7 +8929,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="225" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="225" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A225">
         <v>2048</v>
       </c>
@@ -9033,7 +9034,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="228" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="228" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A228">
         <v>2092</v>
       </c>
@@ -9068,7 +9069,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="229" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="229" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A229">
         <v>2052</v>
       </c>
@@ -9103,7 +9104,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="230" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="230" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A230">
         <v>2267</v>
       </c>
@@ -9138,7 +9139,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="231" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="231" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A231">
         <v>2086</v>
       </c>
@@ -9173,7 +9174,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="232" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="232" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A232">
         <v>2148</v>
       </c>
@@ -9243,7 +9244,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="234" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="234" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A234">
         <v>2026</v>
       </c>
@@ -9278,7 +9279,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="235" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="235" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A235">
         <v>2035</v>
       </c>
@@ -9313,7 +9314,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="236" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="236" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A236">
         <v>2062</v>
       </c>
@@ -9348,7 +9349,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="237" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="237" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A237">
         <v>2292</v>
       </c>
@@ -9383,7 +9384,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="238" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="238" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A238">
         <v>2023</v>
       </c>
@@ -9418,7 +9419,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="239" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="239" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A239">
         <v>2296</v>
       </c>
@@ -9453,7 +9454,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="240" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="240" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A240">
         <v>2177</v>
       </c>
@@ -9488,7 +9489,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="241" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="241" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A241">
         <v>2226</v>
       </c>
@@ -9523,7 +9524,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="242" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="242" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A242">
         <v>2059</v>
       </c>
@@ -9558,7 +9559,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="243" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="243" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A243">
         <v>2021</v>
       </c>
@@ -9628,7 +9629,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="245" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="245" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A245">
         <v>2182</v>
       </c>
@@ -9698,7 +9699,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="247" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="247" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A247">
         <v>2096</v>
       </c>
@@ -9733,7 +9734,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="248" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="248" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A248">
         <v>2283</v>
       </c>
@@ -9768,7 +9769,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="249" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="249" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A249">
         <v>2102</v>
       </c>
@@ -9803,7 +9804,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="250" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="250" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A250">
         <v>2079</v>
       </c>
@@ -9838,7 +9839,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="251" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="251" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A251">
         <v>2169</v>
       </c>
@@ -9873,7 +9874,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="252" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="252" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A252">
         <v>2184</v>
       </c>
@@ -9943,7 +9944,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="254" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="254" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A254">
         <v>2004</v>
       </c>
@@ -9978,7 +9979,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="255" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="255" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A255">
         <v>2074</v>
       </c>
@@ -10013,7 +10014,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="256" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="256" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A256">
         <v>2162</v>
       </c>
@@ -10048,7 +10049,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="257" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="257" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A257">
         <v>2139</v>
       </c>
@@ -10083,7 +10084,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="258" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="258" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A258">
         <v>2272</v>
       </c>
@@ -10153,7 +10154,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="260" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="260" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A260">
         <v>2140</v>
       </c>
@@ -10188,7 +10189,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="261" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="261" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A261">
         <v>2158</v>
       </c>
@@ -10223,7 +10224,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="262" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="262" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A262">
         <v>2200</v>
       </c>
@@ -10258,7 +10259,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="263" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="263" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A263">
         <v>2295</v>
       </c>
@@ -10293,7 +10294,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="264" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="264" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A264">
         <v>2215</v>
       </c>
@@ -10328,7 +10329,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="265" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="265" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A265">
         <v>2129</v>
       </c>
@@ -10363,7 +10364,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="266" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="266" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A266">
         <v>2119</v>
       </c>
@@ -10398,7 +10399,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="267" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="267" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A267">
         <v>2290</v>
       </c>
@@ -10433,7 +10434,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="268" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="268" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A268">
         <v>2150</v>
       </c>
@@ -10468,7 +10469,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="269" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="269" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A269">
         <v>2287</v>
       </c>
@@ -10503,7 +10504,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="270" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="270" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A270">
         <v>2266</v>
       </c>
@@ -10538,7 +10539,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="271" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="271" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A271">
         <v>2178</v>
       </c>
@@ -10573,7 +10574,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="272" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="272" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A272">
         <v>2211</v>
       </c>
@@ -10608,7 +10609,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="273" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="273" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A273">
         <v>2028</v>
       </c>
@@ -10643,7 +10644,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="274" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="274" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A274">
         <v>2237</v>
       </c>
@@ -10678,7 +10679,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="275" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="275" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A275">
         <v>2212</v>
       </c>
@@ -10713,7 +10714,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="276" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="276" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A276">
         <v>2098</v>
       </c>
@@ -10783,7 +10784,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="278" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="278" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A278">
         <v>2280</v>
       </c>
@@ -10818,7 +10819,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="279" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="279" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A279">
         <v>2151</v>
       </c>
@@ -10853,7 +10854,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="280" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="280" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A280">
         <v>2183</v>
       </c>
@@ -10888,7 +10889,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="281" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="281" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A281">
         <v>2189</v>
       </c>
@@ -10923,7 +10924,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="282" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="282" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A282">
         <v>2112</v>
       </c>
@@ -10958,7 +10959,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="283" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="283" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A283">
         <v>2103</v>
       </c>
@@ -10993,7 +10994,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="284" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="284" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A284">
         <v>2107</v>
       </c>
@@ -11028,7 +11029,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="285" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="285" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A285">
         <v>2123</v>
       </c>
@@ -11063,7 +11064,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="286" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="286" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A286">
         <v>2173</v>
       </c>
@@ -11098,7 +11099,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="287" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="287" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A287">
         <v>2033</v>
       </c>
@@ -11133,7 +11134,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="288" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="288" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A288">
         <v>2085</v>
       </c>
@@ -11238,7 +11239,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="291" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="291" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A291">
         <v>2288</v>
       </c>
@@ -11273,7 +11274,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="292" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="292" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A292">
         <v>2273</v>
       </c>
@@ -11308,7 +11309,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="293" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="293" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A293">
         <v>2256</v>
       </c>
@@ -11343,7 +11344,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="294" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="294" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A294">
         <v>2116</v>
       </c>
@@ -11378,7 +11379,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="295" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="295" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A295">
         <v>2186</v>
       </c>
@@ -11413,7 +11414,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="296" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="296" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A296">
         <v>2153</v>
       </c>
@@ -11448,7 +11449,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="297" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="297" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A297">
         <v>2157</v>
       </c>
@@ -11483,7 +11484,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="298" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="298" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A298">
         <v>2106</v>
       </c>
@@ -11518,7 +11519,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="299" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="299" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A299">
         <v>2070</v>
       </c>
@@ -11588,7 +11589,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="301" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="301" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A301">
         <v>2130</v>
       </c>
@@ -11625,6 +11626,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K301" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="East"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:K301">
       <sortCondition ref="D1:D301"/>
     </sortState>

</xml_diff>